<commit_message>
Scrub generator branding from workbook metadata
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/credit-model.xlsx
+++ b/outputs/credit-model.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R6548fbb277aa4c4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rcfac1850bfcd4d5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financials" sheetId="3" r:id="R232b2eb793744acb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liquidity" sheetId="4" r:id="Rda85e0b0da874adc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rating" sheetId="5" r:id="R9f6d214763274201"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collateral" sheetId="6" r:id="Raf76a395913343e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio" sheetId="7" r:id="R2e0ddb0f0b10428c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="8" r:id="R3c68c0b1c7154695"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="9" r:id="Rc5381c3a9dda4514"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditions" sheetId="10" r:id="Rdc73e9feb5dc4c2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Matrix" sheetId="11" r:id="R83cc877d3c924e65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Risks" sheetId="12" r:id="R51ef0b14330f4718"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Covenants" sheetId="13" r:id="Ra7620d3d44004b16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="14" r:id="R1a9e94ac5f144c9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escalations" sheetId="15" r:id="Ra5a9924171f9477c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="16" r:id="R58da7fae2f0b483c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R08a5d826158a4ebc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Ra5b66e7221c54680"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financials" sheetId="3" r:id="R9752cf6242c54cf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liquidity" sheetId="4" r:id="R79b2fb6d16c045f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rating" sheetId="5" r:id="R4864357531ec47cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collateral" sheetId="6" r:id="R729fc98bba99476d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio" sheetId="7" r:id="R4976bce860844a63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="8" r:id="Rd351b3d463ce4c6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="9" r:id="R3eeed1e1ab0d4cc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditions" sheetId="10" r:id="R74b89286679b49bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Matrix" sheetId="11" r:id="R2e2179590507499c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Risks" sheetId="12" r:id="R940925dc9065445e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Covenants" sheetId="13" r:id="Rf2593ef328d54e65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="14" r:id="Ra2bf5f1dd14d448c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escalations" sheetId="15" r:id="R4276c85163f34fd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="16" r:id="R0575116b6ca04fb8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -738,7 +738,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4e8322fd05d54a55"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfea3458ecc754dd4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -748,9 +748,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -800,7 +800,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2447,7 +2447,7 @@
     <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="BLOCKED"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R847e43c1893f4b67"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R501cfe614d804d52"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Release case version 1.1.0 with link previews, social card, and new repo name
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/credit-model.xlsx
+++ b/outputs/credit-model.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R08a5d826158a4ebc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Ra5b66e7221c54680"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financials" sheetId="3" r:id="R9752cf6242c54cf3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liquidity" sheetId="4" r:id="R79b2fb6d16c045f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rating" sheetId="5" r:id="R4864357531ec47cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collateral" sheetId="6" r:id="R729fc98bba99476d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio" sheetId="7" r:id="R4976bce860844a63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="8" r:id="Rd351b3d463ce4c6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="9" r:id="R3eeed1e1ab0d4cc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditions" sheetId="10" r:id="R74b89286679b49bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Matrix" sheetId="11" r:id="R2e2179590507499c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Risks" sheetId="12" r:id="R940925dc9065445e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Covenants" sheetId="13" r:id="Rf2593ef328d54e65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="14" r:id="Ra2bf5f1dd14d448c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escalations" sheetId="15" r:id="R4276c85163f34fd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="16" r:id="R0575116b6ca04fb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="rIdX6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="rIdX7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financials" sheetId="3" r:id="rIdX8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liquidity" sheetId="4" r:id="rIdX9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rating" sheetId="5" r:id="rIdX10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collateral" sheetId="6" r:id="rIdX11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio" sheetId="7" r:id="rIdX12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="8" r:id="rIdX13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="9" r:id="rIdX14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditions" sheetId="10" r:id="rIdX15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Matrix" sheetId="11" r:id="rIdX16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Risks" sheetId="12" r:id="rIdX17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Covenants" sheetId="13" r:id="rIdX18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="14" r:id="rIdX19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escalations" sheetId="15" r:id="rIdX20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="16" r:id="rIdX21"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -738,7 +738,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfea3458ecc754dd4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rIdX2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2447,7 +2447,7 @@
     <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="BLOCKED"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R501cfe614d804d52"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rIdX22"/>
 </x:worksheet>
 </file>
 

</xml_diff>